<commit_message>
docs(xlsx): onglets et en-tetes
</commit_message>
<xml_diff>
--- a/15-gestion-de-projet-budgetisation/budget-picard.xlsx
+++ b/15-gestion-de-projet-budgetisation/budget-picard.xlsx
@@ -9,8 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TJM" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stocks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commande" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outil stocks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appli commande" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transverse" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planning" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
@@ -24,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00&quot; €&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -72,6 +72,11 @@
       <charset val="1"/>
       <family val="0"/>
       <color rgb="FF0000FF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -147,7 +152,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -262,6 +267,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -526,10 +534,11 @@
     <col width="16" customWidth="1" style="19" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="20">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>Budget interne, pas un devis. Marge commerciale non incluse.</t>
+    <row r="1" ht="30" customHeight="1" s="20">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>Budget interne (pas un devis)
+Marge commerciale non incluse</t>
         </is>
       </c>
     </row>
@@ -568,7 +577,7 @@
         </is>
       </c>
       <c r="B4" s="24">
-        <f>Stocks!F28</f>
+        <f>'Outil stocks'!F28</f>
         <v/>
       </c>
       <c r="C4" s="25">
@@ -576,7 +585,7 @@
         <v/>
       </c>
       <c r="D4" s="24">
-        <f>Stocks!F30</f>
+        <f>'Outil stocks'!F30</f>
         <v/>
       </c>
       <c r="E4" s="26">
@@ -591,7 +600,7 @@
         </is>
       </c>
       <c r="B5" s="24">
-        <f>Commande!F50</f>
+        <f>'Appli commande'!F50</f>
         <v/>
       </c>
       <c r="C5" s="25">
@@ -599,7 +608,7 @@
         <v/>
       </c>
       <c r="D5" s="24">
-        <f>Commande!F52</f>
+        <f>'Appli commande'!F52</f>
         <v/>
       </c>
       <c r="E5" s="26">
@@ -691,7 +700,7 @@
         </is>
       </c>
       <c r="C11" s="29">
-        <f>Stocks!C28</f>
+        <f>'Outil stocks'!C28</f>
         <v/>
       </c>
     </row>
@@ -703,7 +712,7 @@
         </is>
       </c>
       <c r="C12" s="29">
-        <f>Commande!C50</f>
+        <f>'Appli commande'!C50</f>
         <v/>
       </c>
     </row>
@@ -732,6 +741,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -749,13 +761,13 @@
   <cols>
     <col width="22" customWidth="1" style="19" min="1" max="1"/>
     <col width="12" customWidth="1" style="19" min="2" max="2"/>
-    <col width="70" customWidth="1" style="19" min="3" max="3"/>
+    <col width="30" customWidth="1" style="19" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="20">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>TJM retenus (€ HT par jour). Cellules bleues = valeurs saisies, à modifier ici.</t>
+    <row r="1" ht="16" customHeight="1" s="20">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>TJM retenus (€ HT par jour)</t>
         </is>
       </c>
     </row>
@@ -788,7 +800,7 @@
       </c>
       <c r="C4" s="23" t="inlineStr">
         <is>
-          <t>Silkhom 2025 CDP confirmé grandes villes 500-650, TJMètre 2026 médian 600</t>
+          <t>Silkhom 2025, TJMètre 2026</t>
         </is>
       </c>
     </row>
@@ -803,7 +815,7 @@
       </c>
       <c r="C5" s="23" t="inlineStr">
         <is>
-          <t>Silkhom 2025 UX/UI confirmé grandes villes 330-450, freelance-informatique 3-4 ans 440</t>
+          <t>Silkhom 2025</t>
         </is>
       </c>
     </row>
@@ -818,7 +830,7 @@
       </c>
       <c r="C6" s="23" t="inlineStr">
         <is>
-          <t>Silkhom 2025 front JS confirmé grandes villes 350-450, haut de fourchette</t>
+          <t>Silkhom 2025</t>
         </is>
       </c>
     </row>
@@ -833,7 +845,7 @@
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>Malt 2026 Symfony 3-7 ans 401, 8-15 ans 523</t>
+          <t>Malt 2026</t>
         </is>
       </c>
     </row>
@@ -848,7 +860,7 @@
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>même base que dev front / back</t>
+          <t>même base que front et back</t>
         </is>
       </c>
     </row>
@@ -863,7 +875,7 @@
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Silkhom 2025 testeur QA confirmé grandes villes 350-450, haut de fourchette</t>
+          <t>Silkhom 2025</t>
         </is>
       </c>
     </row>
@@ -878,7 +890,7 @@
       </c>
       <c r="C10" s="23" t="inlineStr">
         <is>
-          <t>Silkhom 2025 DevOps confirmé grandes villes 450-530, TJMètre 600</t>
+          <t>Silkhom 2025, TJMètre 2026</t>
         </is>
       </c>
     </row>
@@ -893,7 +905,7 @@
       </c>
       <c r="C11" s="23" t="inlineStr">
         <is>
-          <t>Free-Work 665 en direct, donneespersonnelles.fr 800-1200</t>
+          <t>Free-Work</t>
         </is>
       </c>
     </row>
@@ -946,6 +958,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -969,10 +984,12 @@
     <col width="18" customWidth="1" style="19" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="20">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>Outil stocks, grille de coûts par lot. Charge en jours-homme, tâche de 7 j max.</t>
+    <row r="1" ht="44" customHeight="1" s="20">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>Outil stocks, grille de coûts par lot
+Charge en jours-homme
+Tâche de 7 jours max</t>
         </is>
       </c>
     </row>
@@ -1665,6 +1682,9 @@
       <c r="F32" s="23" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1688,10 +1708,12 @@
     <col width="18" customWidth="1" style="19" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="20">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>Appli de commande, grille de coûts par lot. Charge en jours-homme, tâche de 7 j max.</t>
+    <row r="1" ht="44" customHeight="1" s="20">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>Appli de commande, grille de coûts par lot
+Charge en jours-homme
+Tâche de 7 jours max</t>
         </is>
       </c>
     </row>
@@ -2970,6 +2992,9 @@
       <c r="F54" s="23" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2994,10 +3019,12 @@
     <col width="18" customWidth="1" style="19" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="20">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>Postes transverses aux deux projets. Prix hébergement HT (OVHcloud page VPS, sept. 2026), Figma 16 $ pris à 15 €.</t>
+    <row r="1" ht="44" customHeight="1" s="20">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>Postes transverses aux deux projets
+Prix hébergement HT (OVHcloud VPS)
+Figma 16 $ (15 €)</t>
         </is>
       </c>
     </row>
@@ -3485,6 +3512,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3505,10 +3535,12 @@
     <col width="5" customWidth="1" style="19" min="3" max="16"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="20">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>Planning indicatif sur 14 semaines. Une cellule colorée = le lot est actif cette semaine. J = jalon.</t>
+    <row r="1" ht="44" customHeight="1" s="20">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>Planning indicatif sur 14 semaines
+Cellule colorée = lot actif cette semaine
+J = jalon</t>
         </is>
       </c>
     </row>
@@ -4156,6 +4188,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:P1"/>
+  </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>